<commit_message>
converters/DCAT: refresh profile-coverage workbook [generated]
156 of 254 rows now mapped (up from 138) after the Tier/Bucket-B/odrs wiring; 20 wild predicates. Output of make_coverage_xlsx.py.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/converters/DCAT/dcat_profile_coverage.xlsx
+++ b/converters/DCAT/dcat_profile_coverage.xlsx
@@ -9200,7 +9200,11 @@
           <t>odrs:RightsStatement</t>
         </is>
       </c>
-      <c r="C236" s="2" t="inlineStr"/>
+      <c r="C236" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="D236" s="3" t="inlineStr"/>
       <c r="E236" s="3" t="inlineStr"/>
       <c r="F236" s="3" t="inlineStr"/>
@@ -9228,7 +9232,11 @@
           <t>odrs:RightsStatement</t>
         </is>
       </c>
-      <c r="C237" s="2" t="inlineStr"/>
+      <c r="C237" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="D237" s="3" t="inlineStr"/>
       <c r="E237" s="3" t="inlineStr"/>
       <c r="F237" s="3" t="inlineStr"/>
@@ -9256,7 +9264,11 @@
           <t>odrs:RightsStatement</t>
         </is>
       </c>
-      <c r="C238" s="2" t="inlineStr"/>
+      <c r="C238" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="D238" s="3" t="inlineStr"/>
       <c r="E238" s="3" t="inlineStr"/>
       <c r="F238" s="3" t="inlineStr"/>
@@ -9765,7 +9777,7 @@
       </c>
       <c r="B256" s="5" t="n"/>
       <c r="C256" s="6" t="n">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D256" s="6" t="n">
         <v>99</v>

</xml_diff>